<commit_message>
birth reqs table fix
</commit_message>
<xml_diff>
--- a/docs/v2.0.0/CodeSystem-VRM-Status-cs.xlsx
+++ b/docs/v2.0.0/CodeSystem-VRM-Status-cs.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-07-09T11:57:36-04:00</t>
+    <t>2025-08-11T16:10:00-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -171,7 +171,7 @@
     <t>Manual Coding Canceled - Update</t>
   </si>
   <si>
-    <t>An update has been submitted for a death record that is queued for manual coding.  The manual coding
+    <t>An update has been submitted for a death record that is queued for manual coding.  The manual coding
 has been canceled for the original record.</t>
   </si>
   <si>
@@ -181,7 +181,7 @@
     <t>Manual Coding Canceled - Void</t>
   </si>
   <si>
-    <t>A void request has been received for a death record that is queued for manual coding.  The manual coding
+    <t>A void request has been received for a death record that is queued for manual coding.  The manual coding
 has been canceled for the original record.</t>
   </si>
   <si>

</xml_diff>